<commit_message>
Regenerate the Digimock workbook with the corrected priority
The brief now leads with kWh Coffee, BULLITT and CHAI MAMA as TOP MATCH, and
Sami's Superfoods follows as a clearly secondary fourth card. All nine
qualified opportunities remain on the OPPORTUNITIES sheet.

Generated and not sent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017oAcVz7tCdUxv4ef43M9sY
</commit_message>
<xml_diff>
--- a/reports/customer_test/2026-037/LaunchTrace_Food_Digimock_2026-037.xlsx
+++ b/reports/customer_test/2026-037/LaunchTrace_Food_Digimock_2026-037.xlsx
@@ -1037,7 +1037,7 @@
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E8" s="8" t="n"/>
@@ -1099,7 +1099,7 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>LaunchTrace reads the UK Intellectual Property Office trade mark journal every week, matches each food and drink applicant to Companies House, and keeps only the brands that look genuinely early-stage. This brief covers the opportunities from that week that are relevant to what Digimock sells. Every company here has protected a brand name in the last few weeks; none of them has been contacted, and none has asked to be introduced to a supplier.</t>
+          <t>LaunchTrace reads the UK Intellectual Property Office trade mark journal every week, matches each food and drink applicant to Companies House, and keeps only the brands that look genuinely early-stage. This brief covers the opportunities from that week that are relevant to what Digimock sells. Every company here has recently filed a UK trade mark application for a brand or product range; none of them has been contacted, and none has asked to be introduced to a supplier.</t>
         </is>
       </c>
       <c r="C11" s="1" t="n"/>
@@ -1311,7 +1311,7 @@
       <c r="I24" s="20" t="n"/>
       <c r="J24" s="1" t="n"/>
     </row>
-    <row r="25" ht="32" customHeight="1">
+    <row r="25" ht="46" customHeight="1">
       <c r="A25" s="1" t="n"/>
       <c r="B25" s="21" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. kWh Coffee is already selling from its own site, so pack is a live decision rather than a future one.</t>
+          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. The brand is already trading, so this may be more relevant as a range-extension, alternative-supplier or short-run conversation.</t>
         </is>
       </c>
       <c r="D25" s="1" t="n"/>
@@ -1355,7 +1355,7 @@
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>2.  Sami's Superfoods</t>
+          <t>2.  BULLITT</t>
         </is>
       </c>
       <c r="C27" s="13" t="n"/>
@@ -1375,7 +1375,7 @@
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>SAMIS SUPERFOODS LTD  ·  Sheffield  ·  Snacks</t>
+          <t>COLDHARBOUR FOODS LIMITED  ·  Marlow  ·  Cereal, protein and energy bars</t>
         </is>
       </c>
       <c r="C28" s="1" t="n"/>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="C29" s="22" t="inlineStr">
         <is>
-          <t>Nuts — roasted and salted, flavoured, nut butters, snack mixes and dried fruit</t>
+          <t>Energy bars</t>
         </is>
       </c>
       <c r="D29" s="1" t="n"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="C30" s="22" t="inlineStr">
         <is>
-          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 5 years before the filing. Selling direct from its own site, with no multiple-retailer listings found.</t>
+          <t>Filed 27 Aug, published 11 Sep. First trade mark from a company incorporated 6 months before the filing, covering a single product range. No website we could confirm.</t>
         </is>
       </c>
       <c r="D30" s="1" t="n"/>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C31" s="22" t="inlineStr">
         <is>
-          <t>Nuts go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. Sami's Superfoods is already selling from its own site, so pack is a live decision rather than a future one.</t>
+          <t>Energy bars are flow-wrapped, so wrapper film and artwork are part of getting a first production run onto shelf. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="D31" s="1" t="n"/>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C32" s="24" t="inlineStr">
         <is>
-          <t>Resealable printed pouches for the nut and snack-mix range — one short run per flavour rather than one long run.</t>
+          <t>First-run bar wrappers — flow-wrap film at launch quantities.</t>
         </is>
       </c>
       <c r="D32" s="15" t="n"/>
@@ -1471,16 +1471,16 @@
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>3.  BULLITT</t>
+          <t>3.  چاى مامه CHAI MAMA</t>
         </is>
       </c>
       <c r="C33" s="13" t="n"/>
       <c r="D33" s="13" t="n"/>
       <c r="E33" s="13" t="n"/>
       <c r="F33" s="13" t="n"/>
-      <c r="G33" s="25" t="inlineStr">
-        <is>
-          <t>STRONG</t>
+      <c r="G33" s="18" t="inlineStr">
+        <is>
+          <t>TOP MATCH</t>
         </is>
       </c>
       <c r="H33" s="13" t="n"/>
@@ -1491,7 +1491,7 @@
       <c r="A34" s="1" t="n"/>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>COLDHARBOUR FOODS LIMITED  ·  Marlow  ·  Cereal, protein and energy bars</t>
+          <t>FROND FOODS LTD  ·  Liverpool  ·  Coffee, tea and hot drinks</t>
         </is>
       </c>
       <c r="C34" s="1" t="n"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C35" s="22" t="inlineStr">
         <is>
-          <t>Energy bars</t>
+          <t>Tea — loose leaf, tea bags and chai</t>
         </is>
       </c>
       <c r="D35" s="1" t="n"/>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="C36" s="22" t="inlineStr">
         <is>
-          <t>Filed 27 Aug, published 11 Sep. First trade mark from a company incorporated 6 months before the filing, covering a single product range. No website we could confirm.</t>
+          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 10 months before the filing, covering a single product range. No website we could confirm.</t>
         </is>
       </c>
       <c r="D36" s="1" t="n"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C37" s="22" t="inlineStr">
         <is>
-          <t>Energy bars are flow-wrapped. Wrapper film and artwork have to be settled before the first production run, not after it. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Tea is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="D37" s="1" t="n"/>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="C38" s="24" t="inlineStr">
         <is>
-          <t>First-run bar wrappers — flow-wrap film at launch quantities, while the artwork is still open.</t>
+          <t>Small-batch printed tea pouches, with digital print keeping the quantity per SKU low.</t>
         </is>
       </c>
       <c r="D38" s="15" t="n"/>
@@ -1587,7 +1587,7 @@
       <c r="A39" s="1" t="n"/>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>4.  GIGGLECHOC</t>
+          <t>4.  Sami's Superfoods</t>
         </is>
       </c>
       <c r="C39" s="13" t="n"/>
@@ -1607,7 +1607,7 @@
       <c r="A40" s="1" t="n"/>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>JOKE IT LTD  ·  Portsmouth  ·  Confectionery, chocolate and sweets</t>
+          <t>SAMIS SUPERFOODS LTD  ·  Sheffield  ·  Snacks</t>
         </is>
       </c>
       <c r="C40" s="1" t="n"/>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="C41" s="22" t="inlineStr">
         <is>
-          <t>Chocolate — sugar confectionery and dairy confectionery</t>
+          <t>Nuts — roasted and salted, flavoured, nut butters, snack mixes and dried fruit</t>
         </is>
       </c>
       <c r="D41" s="1" t="n"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="C42" s="22" t="inlineStr">
         <is>
-          <t>Filed 28 Aug, published 11 Sep. First trade mark from a company incorporated 8 months before the filing, and the only mark they filed this week. No website we could confirm.</t>
+          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 5 years before the filing. Selling direct from its own site, with no multiple-retailer listings found.</t>
         </is>
       </c>
       <c r="D42" s="1" t="n"/>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="C43" s="22" t="inlineStr">
         <is>
-          <t>Chocolate uses printed film, flow-wrap and pouches. A range that pairs sweets with other merchandise usually carries several small formats rather than one. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Nuts go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. The brand is already trading, so this may be more relevant as a range-extension, alternative-supplier or short-run conversation.</t>
         </is>
       </c>
       <c r="D43" s="1" t="n"/>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="C44" s="24" t="inlineStr">
         <is>
-          <t>Short-run printed film and pouches across a multi-SKU confectionery range, where no single line justifies a long run.</t>
+          <t>Resealable printed pouches for the nut and snack-mix range — one short run per flavour rather than one long run.</t>
         </is>
       </c>
       <c r="D44" s="15" t="n"/>
@@ -1715,7 +1715,7 @@
       <c r="A46" s="1" t="n"/>
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>Suggested sales angles are LaunchTrace's view of how you might approach each brand. They are not requests, enquiries or stated requirements.</t>
+          <t>Suggested sales angles are LaunchTrace's view of how you might approach each brand. They are a suggested approach, not evidence of current buying intent, and not a request, enquiry or stated requirement.</t>
         </is>
       </c>
       <c r="C46" s="1" t="n"/>
@@ -1923,7 +1923,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>Suggested sales angles are LaunchTrace's view of how you might approach each brand. They are not requests, enquiries or stated requirements.</t>
+          <t>Suggested sales angles are LaunchTrace's view of how you might approach each brand. They are a suggested approach, not evidence of current buying intent, and not a request, enquiry or stated requirement.</t>
         </is>
       </c>
       <c r="B3" s="1" t="n"/>
@@ -2036,7 +2036,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="68" customHeight="1">
+    <row r="5" ht="80" customHeight="1">
       <c r="A5" s="32" t="inlineStr">
         <is>
           <t>TOP MATCH</t>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="I5" s="35" t="inlineStr">
         <is>
-          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. kWh Coffee is already selling from its own site, so pack is a live decision rather than a future one.</t>
+          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. The brand is already trading, so this may be more relevant as a range-extension, alternative-supplier or short-run conversation.</t>
         </is>
       </c>
       <c r="J5" s="35" t="inlineStr">
@@ -2120,66 +2120,66 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>Sami's Superfoods</t>
+          <t>BULLITT</t>
         </is>
       </c>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>SAMIS SUPERFOODS LTD</t>
+          <t>COLDHARBOUR FOODS LIMITED</t>
         </is>
       </c>
       <c r="D6" s="34" t="inlineStr">
         <is>
-          <t>Sheffield</t>
+          <t>Marlow</t>
         </is>
       </c>
       <c r="E6" s="34" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Cereal, protein and energy bars</t>
         </is>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
-          <t>Nuts — roasted and salted, flavoured, nut butters, snack mixes and dried fruit</t>
+          <t>Energy bars</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>Early launch</t>
+          <t>Not determined</t>
         </is>
       </c>
       <c r="H6" s="35" t="inlineStr">
         <is>
-          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 5 years before the filing. Selling direct from its own site, with no multiple-retailer listings found.</t>
+          <t>Filed 27 Aug, published 11 Sep. First trade mark from a company incorporated 6 months before the filing, covering a single product range. No website we could confirm.</t>
         </is>
       </c>
       <c r="I6" s="35" t="inlineStr">
         <is>
-          <t>Nuts go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. Sami's Superfoods is already selling from its own site, so pack is a live decision rather than a future one.</t>
+          <t>Energy bars are flow-wrapped, so wrapper film and artwork are part of getting a first production run onto shelf. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="J6" s="35" t="inlineStr">
         <is>
-          <t>Resealable printed pouches for the nut and snack-mix range — one short run per flavour rather than one long run.</t>
-        </is>
-      </c>
-      <c r="K6" s="36" t="inlineStr">
-        <is>
-          <t>samissuperfoods.com</t>
+          <t>First-run bar wrappers — flow-wrap film at launch quantities.</t>
+        </is>
+      </c>
+      <c r="K6" s="39" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="L6" s="36" t="inlineStr">
         <is>
-          <t>UK00004435509</t>
+          <t>UK00004437089</t>
         </is>
       </c>
       <c r="M6" s="36" t="inlineStr">
         <is>
-          <t>13274599</t>
+          <t>17035779</t>
         </is>
       </c>
       <c r="N6" s="37" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="O6" s="37" t="n">
         <v>46276</v>
@@ -2189,24 +2189,24 @@
       <c r="R6" s="38" t="n"/>
     </row>
     <row r="7" ht="68" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>STRONG</t>
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>TOP MATCH</t>
         </is>
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Rose &amp; Grind</t>
+          <t>چاى مامه CHAI MAMA</t>
         </is>
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>ROSE &amp; GRIND LTD</t>
+          <t>FROND FOODS LTD</t>
         </is>
       </c>
       <c r="D7" s="34" t="inlineStr">
         <is>
-          <t>Darlington</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="E7" s="34" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
-          <t>Coffee — whole bean, ground, coffee bags, pods and capsules</t>
+          <t>Tea — loose leaf, tea bags and chai</t>
         </is>
       </c>
       <c r="G7" s="34" t="inlineStr">
@@ -2226,17 +2226,17 @@
       </c>
       <c r="H7" s="35" t="inlineStr">
         <is>
-          <t>Filed 20 Aug, published 11 Sep. First trade mark from a company incorporated in the same month as the filing, covering a single product range. No website we could confirm.</t>
+          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 10 months before the filing, covering a single product range. No website we could confirm.</t>
         </is>
       </c>
       <c r="I7" s="35" t="inlineStr">
         <is>
-          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Tea is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="J7" s="35" t="inlineStr">
         <is>
-          <t>Short-run printed coffee pouches across multiple SKUs, with drip-bag and coffee-bag film as a natural second format.</t>
+          <t>Small-batch printed tea pouches, with digital print keeping the quantity per SKU low.</t>
         </is>
       </c>
       <c r="K7" s="39" t="inlineStr">
@@ -2246,16 +2246,16 @@
       </c>
       <c r="L7" s="36" t="inlineStr">
         <is>
-          <t>UK00004433315</t>
+          <t>UK00004435320</t>
         </is>
       </c>
       <c r="M7" s="36" t="inlineStr">
         <is>
-          <t>17410336</t>
+          <t>16798042</t>
         </is>
       </c>
       <c r="N7" s="37" t="n">
-        <v>46254</v>
+        <v>46259</v>
       </c>
       <c r="O7" s="37" t="n">
         <v>46276</v>
@@ -2272,62 +2272,62 @@
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>چاى مامه CHAI MAMA</t>
+          <t>Sami's Superfoods</t>
         </is>
       </c>
       <c r="C8" s="34" t="inlineStr">
         <is>
-          <t>FROND FOODS LTD</t>
+          <t>SAMIS SUPERFOODS LTD</t>
         </is>
       </c>
       <c r="D8" s="34" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Sheffield</t>
         </is>
       </c>
       <c r="E8" s="34" t="inlineStr">
         <is>
-          <t>Coffee, tea and hot drinks</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
-          <t>Tea — loose leaf, tea bags and chai</t>
+          <t>Nuts — roasted and salted, flavoured, nut butters, snack mixes and dried fruit</t>
         </is>
       </c>
       <c r="G8" s="34" t="inlineStr">
         <is>
-          <t>Not determined</t>
+          <t>Early launch</t>
         </is>
       </c>
       <c r="H8" s="35" t="inlineStr">
         <is>
-          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 10 months before the filing, covering a single product range. No website we could confirm.</t>
+          <t>Filed 25 Aug, published 11 Sep. First trade mark from a company incorporated 5 years before the filing. Selling direct from its own site, with no multiple-retailer listings found.</t>
         </is>
       </c>
       <c r="I8" s="35" t="inlineStr">
         <is>
-          <t>Tea is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Nuts go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. The brand is already trading, so this may be more relevant as a range-extension, alternative-supplier or short-run conversation.</t>
         </is>
       </c>
       <c r="J8" s="35" t="inlineStr">
         <is>
-          <t>Small-batch printed tea pouches, with digital print keeping the quantity per SKU low while the range settles.</t>
-        </is>
-      </c>
-      <c r="K8" s="39" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
+          <t>Resealable printed pouches for the nut and snack-mix range — one short run per flavour rather than one long run.</t>
+        </is>
+      </c>
+      <c r="K8" s="36" t="inlineStr">
+        <is>
+          <t>samissuperfoods.com</t>
         </is>
       </c>
       <c r="L8" s="36" t="inlineStr">
         <is>
-          <t>UK00004435320</t>
+          <t>UK00004435509</t>
         </is>
       </c>
       <c r="M8" s="36" t="inlineStr">
         <is>
-          <t>16798042</t>
+          <t>13274599</t>
         </is>
       </c>
       <c r="N8" s="37" t="n">
@@ -2340,7 +2340,7 @@
       <c r="Q8" s="38" t="n"/>
       <c r="R8" s="38" t="n"/>
     </row>
-    <row r="9" ht="55" customHeight="1">
+    <row r="9" ht="68" customHeight="1">
       <c r="A9" s="33" t="inlineStr">
         <is>
           <t>STRONG</t>
@@ -2348,27 +2348,27 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>BULLITT</t>
+          <t>Rose &amp; Grind</t>
         </is>
       </c>
       <c r="C9" s="34" t="inlineStr">
         <is>
-          <t>COLDHARBOUR FOODS LIMITED</t>
+          <t>ROSE &amp; GRIND LTD</t>
         </is>
       </c>
       <c r="D9" s="34" t="inlineStr">
         <is>
-          <t>Marlow</t>
+          <t>Darlington</t>
         </is>
       </c>
       <c r="E9" s="34" t="inlineStr">
         <is>
-          <t>Cereal, protein and energy bars</t>
+          <t>Coffee, tea and hot drinks</t>
         </is>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
-          <t>Energy bars</t>
+          <t>Coffee — whole bean, ground, coffee bags, pods and capsules</t>
         </is>
       </c>
       <c r="G9" s="34" t="inlineStr">
@@ -2378,17 +2378,17 @@
       </c>
       <c r="H9" s="35" t="inlineStr">
         <is>
-          <t>Filed 27 Aug, published 11 Sep. First trade mark from a company incorporated 6 months before the filing, covering a single product range. No website we could confirm.</t>
+          <t>Filed 20 Aug, published 11 Sep. First trade mark from a company incorporated in the same month as the filing, covering a single product range. No website we could confirm.</t>
         </is>
       </c>
       <c r="I9" s="35" t="inlineStr">
         <is>
-          <t>Energy bars are flow-wrapped. Wrapper film and artwork have to be settled before the first production run, not after it. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Coffee is a printed-pouch category. Film and bag formats are normally the first pack decision a hot-drinks brand makes, and usually across several SKUs at once. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="J9" s="35" t="inlineStr">
         <is>
-          <t>First-run bar wrappers — flow-wrap film at launch quantities, while the artwork is still open.</t>
+          <t>Short-run printed coffee pouches across multiple SKUs, with drip-bag and coffee-bag film as a natural second format.</t>
         </is>
       </c>
       <c r="K9" s="39" t="inlineStr">
@@ -2398,16 +2398,16 @@
       </c>
       <c r="L9" s="36" t="inlineStr">
         <is>
-          <t>UK00004437089</t>
+          <t>UK00004433315</t>
         </is>
       </c>
       <c r="M9" s="36" t="inlineStr">
         <is>
-          <t>17035779</t>
+          <t>17410336</t>
         </is>
       </c>
       <c r="N9" s="37" t="n">
-        <v>46261</v>
+        <v>46254</v>
       </c>
       <c r="O9" s="37" t="n">
         <v>46276</v>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="I10" s="35" t="inlineStr">
         <is>
-          <t>Chocolate uses printed film, flow-wrap and pouches. A range that pairs sweets with other merchandise usually carries several small formats rather than one. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Chocolate uses printed film, flow-wrap and pouches. A range that pairs sweets with other merchandise usually carries several small formats rather than one. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="J10" s="35" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="I11" s="35" t="inlineStr">
         <is>
-          <t>Vegetable crisps and fries go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. There is no brand site we could confirm, so the pack format is likely still open.</t>
+          <t>Vegetable crisps and fries go to market in printed bags and pouches. A range with several variants means several designs, each at modest volume. We could not confirm a brand website, so there is less public evidence about how far the launch has progressed.</t>
         </is>
       </c>
       <c r="J11" s="35" t="inlineStr">
@@ -2568,7 +2568,7 @@
       <c r="Q11" s="38" t="n"/>
       <c r="R11" s="38" t="n"/>
     </row>
-    <row r="12" ht="68" customHeight="1">
+    <row r="12" ht="80" customHeight="1">
       <c r="A12" s="40" t="inlineStr">
         <is>
           <t>RELEVANT</t>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="H12" s="35" t="inlineStr">
         <is>
-          <t>Filed 29 Aug, published 11 Sep. First trade mark from a company incorporated 3 months before the filing, covering a single product range. No website we could confirm, and the signals read pre-launch.</t>
+          <t>Filed 29 Aug, published 11 Sep. First trade mark from a company incorporated 3 months before the filing, covering a single product range. No website we could confirm, and the available signals suggest it is still early in its launch.</t>
         </is>
       </c>
       <c r="I12" s="35" t="inlineStr">
         <is>
-          <t>Yoghurt and dairy is mostly pots and labels rather than film. The granola, frozen and lidding formats in the same filing are the part that is flexible-pack work. The signals read pre-launch, so nothing is likely to be committed yet.</t>
+          <t>Yoghurt and dairy is mostly pots and labels rather than film. The granola, frozen and lidding formats in the same filing are the part that is flexible-pack work. There is little public evidence about the brand so far, so an early introduction is more about being known to them than about any specific project.</t>
         </is>
       </c>
       <c r="J12" s="35" t="inlineStr">
@@ -2644,7 +2644,7 @@
       <c r="Q12" s="38" t="n"/>
       <c r="R12" s="38" t="n"/>
     </row>
-    <row r="13" ht="68" customHeight="1">
+    <row r="13" ht="80" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <t>RELEVANT</t>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="H13" s="35" t="inlineStr">
         <is>
-          <t>Filed 26 Aug, published 11 Sep. First trade mark from a company incorporated 16 months before the filing, covering a single product range. No website we could confirm, and the signals read pre-launch.</t>
+          <t>Filed 26 Aug, published 11 Sep. First trade mark from a company incorporated 16 months before the filing, covering a single product range. No website we could confirm, and the available signals suggest it is still early in its launch.</t>
         </is>
       </c>
       <c r="I13" s="35" t="inlineStr">
         <is>
-          <t>Spices and seasonings reach shelf in glass or in pouches and sachets. Where a brand chooses pouches, it is flexible-pack work from the first batch onwards. The signals read pre-launch, so nothing is likely to be committed yet.</t>
+          <t>Spices and seasonings reach shelf in glass or in pouches and sachets. Where a brand chooses pouches, it is flexible-pack work from the first batch onwards. There is little public evidence about the brand so far, so an early introduction is more about being known to them than about any specific project.</t>
         </is>
       </c>
       <c r="J13" s="35" t="inlineStr">
@@ -2809,11 +2809,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId11"/>
@@ -2947,11 +2947,11 @@
       <c r="G6" s="1" t="n"/>
       <c r="H6" s="1" t="n"/>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="74" customHeight="1">
       <c r="A7" s="1" t="n"/>
       <c r="B7" s="44" t="inlineStr">
         <is>
-          <t>Every week the UK Intellectual Property Office publishes the trade marks that have been filed. A new food or drink brand almost always protects its name before it goes on sale. LaunchTrace reads that journal, works out which applicants are real UK food businesses, checks them against Companies House, and keeps only the ones that look like they are still building rather than already established. What you get is a list of brands at the point where their suppliers have not been chosen yet.</t>
+          <t>Every week the UK Intellectual Property Office publishes the trade mark applications that have been filed. A new food or drink brand almost always files an application for its name before it goes on sale. Publication means the application has been filed and advertised, not that registration is complete. LaunchTrace reads that journal, works out which applicants are real UK food businesses, checks them against Companies House, and keeps only the ones that look like they are still building rather than already established. What you get is a list of brands early enough in their life to be worth introducing yourself to.</t>
         </is>
       </c>
       <c r="C7" s="1" t="n"/>
@@ -2985,11 +2985,11 @@
       <c r="G9" s="1" t="n"/>
       <c r="H9" s="1" t="n"/>
     </row>
-    <row r="10" ht="46" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="44" t="inlineStr">
         <is>
-          <t>It is the timing evidence: when the name was filed and published, how recently the company behind it was formed, whether this is the first mark we have seen from them, and whether the brand has a website or retailer listings yet. It explains why this week is a sensible moment to make contact, rather than six months from now.</t>
+          <t>It is the timing evidence: when the application was filed and published, how recently the company behind it was formed, whether this is the first mark we have seen from them, and whether the brand has a website or retailer listings yet. It explains why this week is a sensible moment to make contact, rather than six months from now. It does not tell you anything about who they buy from, or what they have already ordered — we have no visibility of that.</t>
         </is>
       </c>
       <c r="C10" s="1" t="n"/>
@@ -3065,7 +3065,7 @@
       <c r="A16" s="1" t="n"/>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t>The angle is our read on what this kind of brand, at this stage, usually needs from a supplier like you. It is a starting point for a first conversation — a sensible opening line and a reason to call — not a statement that the company has asked for that product. Check it against what you actually see on their website or filing before you use it.</t>
+          <t>The angle is our read on what a supplier like you might be able to offer a brand at this stage. It is a starting point for a first conversation — a sensible opening line and a reason to call — not a statement that the company has asked for that product, and not evidence that any supplier decision is still open. Check it against what you actually see on their website or filing before you use it.</t>
         </is>
       </c>
       <c r="C16" s="1" t="n"/>
@@ -3137,11 +3137,11 @@
       <c r="G21" s="1" t="n"/>
       <c r="H21" s="1" t="n"/>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="74" customHeight="1">
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="44" t="inlineStr">
         <is>
-          <t>TOP MATCH — the strongest launch signals of the week and a direct fit for what you sell. Start here. STRONG — a clear early-stage brand in a category you serve; worth a call this week. RELEVANT — qualified and in scope, but a partial fit; read the suggested angle before spending time on it. Priority combines how early-stage the brand looks with how closely its category matches your business, so it is specific to you and not a general ranking.</t>
+          <t>TOP MATCH — one of the strongest opportunities for you this week. Start here. STRONG — a clear early-stage brand in a category you serve; worth a call this week. RELEVANT — qualified and in scope, but a partial fit; read the suggested angle before spending time on it. Priority is specific to your business, not a general ranking: it weighs how early-stage the brand looks together with how closely what it is launching matches what you sell. A brand can be an unusually strong launch signal in general and still not be one of your best leads, and Priority reflects your side of that.</t>
         </is>
       </c>
       <c r="C22" s="1" t="n"/>

</xml_diff>